<commit_message>
Excel certs sheet and improved server code
</commit_message>
<xml_diff>
--- a/List of Certifications required.xlsx
+++ b/List of Certifications required.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mohammed.saleem\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\imole.adebayo\Desktop\Hackathon\Hackathon-Emad-Luqman-Imole\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B8C23A63-D2E9-4957-AF26-55E143E592AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FA16484-5F19-4DE7-9AC0-C707958F9A9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{8CD59AFF-A47D-483E-8502-065F5E95F4C1}"/>
   </bookViews>
@@ -33,6 +33,299 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="96">
+  <si>
+    <t xml:space="preserve">No. </t>
+  </si>
+  <si>
+    <t>Certification</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Issuing body </t>
+  </si>
+  <si>
+    <t>Link to issuing body Website</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Business analyst </t>
+  </si>
+  <si>
+    <t>BCS: International Diploma in Business Analysis</t>
+  </si>
+  <si>
+    <t>BCS</t>
+  </si>
+  <si>
+    <t>https://www.bcs.org/qualifications-and-certifications/</t>
+  </si>
+  <si>
+    <t>IIBA: CBAP (Certified Business Analysis Professional)</t>
+  </si>
+  <si>
+    <t>IIBA</t>
+  </si>
+  <si>
+    <t>https://www.iiba.org/business-analysis-certifications/</t>
+  </si>
+  <si>
+    <t>Foundation Certificate in Data Protection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Business analyst + Project manager </t>
+  </si>
+  <si>
+    <t>IAPP: CIPP/E</t>
+  </si>
+  <si>
+    <t>IAPP</t>
+  </si>
+  <si>
+    <t>https://iapp.org/certify/</t>
+  </si>
+  <si>
+    <t>Certificate in Business Data Analytics (CBDA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Project manager </t>
+  </si>
+  <si>
+    <t>Professional Scrum Master (PSM I/II)</t>
+  </si>
+  <si>
+    <t>Scrum.org</t>
+  </si>
+  <si>
+    <t>https://www.scrum.org/certifications</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> BCS Foundation/Practitioner Certificate in Data Protection</t>
+  </si>
+  <si>
+    <t>BCS: Foundation Certificate in Data Protection</t>
+  </si>
+  <si>
+    <t>Data engineer</t>
+  </si>
+  <si>
+    <t>AWS Certified Data Engineer ( Associate)</t>
+  </si>
+  <si>
+    <t>AWS</t>
+  </si>
+  <si>
+    <t>https://aws.amazon.com/certification/certified-data-engineer-associate/</t>
+  </si>
+  <si>
+    <t>DP-203: Microsoft Certified: Azure Data Engineer Associate</t>
+  </si>
+  <si>
+    <t>Microsoft</t>
+  </si>
+  <si>
+    <t>https://learn.microsoft.com/en-us/credentials/certifications/</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Google Professional Data Engineer</t>
+  </si>
+  <si>
+    <t>Google Cloud</t>
+  </si>
+  <si>
+    <t>https://cloud.google.com/learn/certification/</t>
+  </si>
+  <si>
+    <t>dbt Analytics Engineering Certification</t>
+  </si>
+  <si>
+    <t>dbt Labs</t>
+  </si>
+  <si>
+    <t>https://www.google.com/search?q=https://www.getdbt.com/certifications/</t>
+  </si>
+  <si>
+    <t>Astronomer Certification for Apache Airflow</t>
+  </si>
+  <si>
+    <t>Astronomer</t>
+  </si>
+  <si>
+    <t>https://www.astronomer.io/certification/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delivery operations manager </t>
+  </si>
+  <si>
+    <t>Professional Scrum Master</t>
+  </si>
+  <si>
+    <t>Professional Scrum Product Owner (PSPO)</t>
+  </si>
+  <si>
+    <t>Certified SAFe® Release Train Engineer (RTE)</t>
+  </si>
+  <si>
+    <t>Scaled Agile</t>
+  </si>
+  <si>
+    <t>https://www.google.com/search?q=https://scaledagile.com/training/</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Kanban Management Professional (KMP)</t>
+  </si>
+  <si>
+    <t>Kanban Univ.</t>
+  </si>
+  <si>
+    <t>https://kanban.university/</t>
+  </si>
+  <si>
+    <t>ITIL 4: ITIL 4 Specialist</t>
+  </si>
+  <si>
+    <t>PeopleCert</t>
+  </si>
+  <si>
+    <t>https://www.peoplecert.org/</t>
+  </si>
+  <si>
+    <t>DevOPs / Platform Engineer</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Google Professional Cloud DevOps Engineer</t>
+  </si>
+  <si>
+    <t>AWS Certified DevOps Engineer – Professional</t>
+  </si>
+  <si>
+    <t>https://aws.amazon.com/certification/</t>
+  </si>
+  <si>
+    <t>AZ-400: Designing and Implementing Microsoft DevOps Solutions</t>
+  </si>
+  <si>
+    <t>CKA (Certified Kubernetes Administrator)</t>
+  </si>
+  <si>
+    <t>CNCF/LF</t>
+  </si>
+  <si>
+    <t>https://training.linuxfoundation.org/certification/</t>
+  </si>
+  <si>
+    <t>CKAD (Certified Kubernetes Application Developer)</t>
+  </si>
+  <si>
+    <t>Terraform Associate (003)</t>
+  </si>
+  <si>
+    <t>HashiCorp</t>
+  </si>
+  <si>
+    <t>https://www.hashicorp.com/certification/</t>
+  </si>
+  <si>
+    <t>IT support Helpdesk</t>
+  </si>
+  <si>
+    <t>CompTIA: A+ (Core 1 &amp; 2)</t>
+  </si>
+  <si>
+    <t>CompTIA</t>
+  </si>
+  <si>
+    <t>https://www.google.com/search?q=https://www.comptia.org/certifications/</t>
+  </si>
+  <si>
+    <t>CompTIA: Tech+ (formerly IT Fundamentals+)</t>
+  </si>
+  <si>
+    <t>Google: IT Support Professional Certificate</t>
+  </si>
+  <si>
+    <t>https://grow.google/certificates/</t>
+  </si>
+  <si>
+    <t>Microsoft: MS-900 (Microsoft 365 Fundamentals)</t>
+  </si>
+  <si>
+    <t>Microsoft: MD-102 (Endpoint Administrator)</t>
+  </si>
+  <si>
+    <t>CCT (Cisco Certified Technician)</t>
+  </si>
+  <si>
+    <t>Cisco</t>
+  </si>
+  <si>
+    <t>https://www.google.com/search?q=https://www.cisco.com/c/en/us/training-events/training-certifications/</t>
+  </si>
+  <si>
+    <t>Software engineer</t>
+  </si>
+  <si>
+    <t>Oracle: Certified Professional: Java SE Developer</t>
+  </si>
+  <si>
+    <t>Oracle</t>
+  </si>
+  <si>
+    <t>https://www.google.com/search?q=https://education.oracle.com/certification/</t>
+  </si>
+  <si>
+    <t>Front-End/Back-End Developer Professional Certificates</t>
+  </si>
+  <si>
+    <t>Meta/IBM</t>
+  </si>
+  <si>
+    <t>https://www.coursera.org/</t>
+  </si>
+  <si>
+    <t>PCPP (Certified Professional in Python Programming)</t>
+  </si>
+  <si>
+    <t>OpenEDG</t>
+  </si>
+  <si>
+    <t>https://www.google.com/search?q=https://pythoninstitute.org/certification/</t>
+  </si>
+  <si>
+    <t>AWS: Certified Developer – Associate (DVA-C02)</t>
+  </si>
+  <si>
+    <t>Azure: AZ-204: Developing Solutions for Microsoft Azure.</t>
+  </si>
+  <si>
+    <t>GCP: Professional Cloud Developer.</t>
+  </si>
+  <si>
+    <t>Test Analyst</t>
+  </si>
+  <si>
+    <t>BCS Practitioner Certificate in Enterprise and Solutions Architecture</t>
+  </si>
+  <si>
+    <t>ISTQB: Certified Tester Foundation Level (v4.0)</t>
+  </si>
+  <si>
+    <t>ISTQB</t>
+  </si>
+  <si>
+    <t>https://www.istqb.org/certifications/</t>
+  </si>
+  <si>
+    <t>ISTQB: Agile Tester Extension</t>
+  </si>
+  <si>
+    <t>BCS: Foundation Certificate in Software Testing</t>
+  </si>
+  <si>
+    <t>ISTQB: AI Testing (CT-AI)</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -402,9 +695,612 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F136C923-7755-4332-B205-608D8C676040}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:K43"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" t="s">
+        <v>2</v>
+      </c>
+      <c r="K1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" t="s">
+        <v>6</v>
+      </c>
+      <c r="K2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3" t="s">
+        <v>9</v>
+      </c>
+      <c r="K3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" t="s">
+        <v>14</v>
+      </c>
+      <c r="K5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" t="s">
+        <v>9</v>
+      </c>
+      <c r="K6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G7" t="s">
+        <v>19</v>
+      </c>
+      <c r="K7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G8" t="s">
+        <v>6</v>
+      </c>
+      <c r="K8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" t="s">
+        <v>22</v>
+      </c>
+      <c r="G9" t="s">
+        <v>6</v>
+      </c>
+      <c r="K9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" t="s">
+        <v>24</v>
+      </c>
+      <c r="G10" t="s">
+        <v>25</v>
+      </c>
+      <c r="K10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G11" t="s">
+        <v>28</v>
+      </c>
+      <c r="K11" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" t="s">
+        <v>30</v>
+      </c>
+      <c r="G12" t="s">
+        <v>31</v>
+      </c>
+      <c r="K12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" t="s">
+        <v>33</v>
+      </c>
+      <c r="G13" t="s">
+        <v>34</v>
+      </c>
+      <c r="K13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" t="s">
+        <v>36</v>
+      </c>
+      <c r="G14" t="s">
+        <v>37</v>
+      </c>
+      <c r="K14" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" t="s">
+        <v>40</v>
+      </c>
+      <c r="G15" t="s">
+        <v>19</v>
+      </c>
+      <c r="K15" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" t="s">
+        <v>41</v>
+      </c>
+      <c r="G16" t="s">
+        <v>19</v>
+      </c>
+      <c r="K16" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>39</v>
+      </c>
+      <c r="B17" t="s">
+        <v>42</v>
+      </c>
+      <c r="G17" t="s">
+        <v>43</v>
+      </c>
+      <c r="K17" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>39</v>
+      </c>
+      <c r="B18" t="s">
+        <v>45</v>
+      </c>
+      <c r="G18" t="s">
+        <v>46</v>
+      </c>
+      <c r="K18" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>39</v>
+      </c>
+      <c r="B19" t="s">
+        <v>48</v>
+      </c>
+      <c r="G19" t="s">
+        <v>49</v>
+      </c>
+      <c r="K19" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>51</v>
+      </c>
+      <c r="B20" t="s">
+        <v>52</v>
+      </c>
+      <c r="G20" t="s">
+        <v>31</v>
+      </c>
+      <c r="K20" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>51</v>
+      </c>
+      <c r="B21" t="s">
+        <v>53</v>
+      </c>
+      <c r="G21" t="s">
+        <v>25</v>
+      </c>
+      <c r="K21" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>51</v>
+      </c>
+      <c r="B22" t="s">
+        <v>55</v>
+      </c>
+      <c r="G22" t="s">
+        <v>28</v>
+      </c>
+      <c r="K22" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>51</v>
+      </c>
+      <c r="B23" t="s">
+        <v>56</v>
+      </c>
+      <c r="G23" t="s">
+        <v>57</v>
+      </c>
+      <c r="K23" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>51</v>
+      </c>
+      <c r="B24" t="s">
+        <v>59</v>
+      </c>
+      <c r="G24" t="s">
+        <v>57</v>
+      </c>
+      <c r="K24" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>51</v>
+      </c>
+      <c r="B25" t="s">
+        <v>60</v>
+      </c>
+      <c r="G25" t="s">
+        <v>61</v>
+      </c>
+      <c r="K25" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>63</v>
+      </c>
+      <c r="B26" t="s">
+        <v>64</v>
+      </c>
+      <c r="G26" t="s">
+        <v>65</v>
+      </c>
+      <c r="K26" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>63</v>
+      </c>
+      <c r="B27" t="s">
+        <v>67</v>
+      </c>
+      <c r="G27" t="s">
+        <v>65</v>
+      </c>
+      <c r="K27" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>63</v>
+      </c>
+      <c r="B28" t="s">
+        <v>68</v>
+      </c>
+      <c r="G28" t="s">
+        <v>31</v>
+      </c>
+      <c r="K28" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>63</v>
+      </c>
+      <c r="B29" t="s">
+        <v>70</v>
+      </c>
+      <c r="G29" t="s">
+        <v>28</v>
+      </c>
+      <c r="K29" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>63</v>
+      </c>
+      <c r="B30" t="s">
+        <v>71</v>
+      </c>
+      <c r="G30" t="s">
+        <v>28</v>
+      </c>
+      <c r="K30" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>63</v>
+      </c>
+      <c r="B31" t="s">
+        <v>72</v>
+      </c>
+      <c r="G31" t="s">
+        <v>73</v>
+      </c>
+      <c r="K31" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>75</v>
+      </c>
+      <c r="B32" t="s">
+        <v>76</v>
+      </c>
+      <c r="G32" t="s">
+        <v>77</v>
+      </c>
+      <c r="K32" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>75</v>
+      </c>
+      <c r="B33" t="s">
+        <v>79</v>
+      </c>
+      <c r="G33" t="s">
+        <v>80</v>
+      </c>
+      <c r="K33" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>75</v>
+      </c>
+      <c r="B34" t="s">
+        <v>82</v>
+      </c>
+      <c r="G34" t="s">
+        <v>83</v>
+      </c>
+      <c r="K34" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>75</v>
+      </c>
+      <c r="B35" t="s">
+        <v>85</v>
+      </c>
+      <c r="G35" t="s">
+        <v>25</v>
+      </c>
+      <c r="K35" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>75</v>
+      </c>
+      <c r="B36" t="s">
+        <v>86</v>
+      </c>
+      <c r="G36" t="s">
+        <v>28</v>
+      </c>
+      <c r="K36" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>75</v>
+      </c>
+      <c r="B37" t="s">
+        <v>87</v>
+      </c>
+      <c r="G37" t="s">
+        <v>31</v>
+      </c>
+      <c r="K37" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>88</v>
+      </c>
+      <c r="B38" t="s">
+        <v>89</v>
+      </c>
+      <c r="G38" t="s">
+        <v>6</v>
+      </c>
+      <c r="K38" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>88</v>
+      </c>
+      <c r="B39" t="s">
+        <v>90</v>
+      </c>
+      <c r="G39" t="s">
+        <v>91</v>
+      </c>
+      <c r="K39" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>88</v>
+      </c>
+      <c r="B40" t="s">
+        <v>93</v>
+      </c>
+      <c r="G40" t="s">
+        <v>91</v>
+      </c>
+      <c r="K40" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>88</v>
+      </c>
+      <c r="B41" t="s">
+        <v>94</v>
+      </c>
+      <c r="G41" t="s">
+        <v>6</v>
+      </c>
+      <c r="K41" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>88</v>
+      </c>
+      <c r="B42" t="s">
+        <v>95</v>
+      </c>
+      <c r="G42" t="s">
+        <v>91</v>
+      </c>
+      <c r="K42" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>88</v>
+      </c>
+      <c r="B43" t="s">
+        <v>22</v>
+      </c>
+      <c r="G43" t="s">
+        <v>6</v>
+      </c>
+      <c r="K43" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>